<commit_message>
Updated deprecated functions - C++ on Linux workbook (removed extra sheet) [distribution tree]
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/working_material/deprecated functions/deprecated functions - C++ on Linux.xlsx
+++ b/distribution/reference_documents/working_material/deprecated functions/deprecated functions - C++ on Linux.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/deprecated functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328A20DF-C1DA-0A47-BF52-35F1CFA5A69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C07F6B9-27DD-0142-A66E-AFFFAD35BEB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18020" yWindow="8600" windowWidth="34700" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-79100" yWindow="-39000" windowWidth="30240" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cover sheet" sheetId="10" r:id="rId1"/>
@@ -19,8 +19,7 @@
     <sheet name="Format" sheetId="5" r:id="rId4"/>
     <sheet name="Memory" sheetId="3" r:id="rId5"/>
     <sheet name="Strings" sheetId="11" r:id="rId6"/>
-    <sheet name="Sheet1" sheetId="13" r:id="rId7"/>
-    <sheet name="Time" sheetId="12" r:id="rId8"/>
+    <sheet name="Time" sheetId="12" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -43,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="150">
   <si>
     <t>Deprecated Functions</t>
   </si>
@@ -952,6 +951,9 @@
   </si>
   <si>
     <t>fmt</t>
+  </si>
+  <si>
+    <t>removed extra sheet</t>
   </si>
 </sst>
 </file>
@@ -1341,6 +1343,19 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1350,32 +1365,19 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="24" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1723,18 +1725,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="63">
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="50"/>
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
     </row>
     <row r="3" spans="2:11">
       <c r="B3" s="9"/>
@@ -1746,119 +1748,119 @@
         <v>1</v>
       </c>
       <c r="C4" s="11"/>
-      <c r="D4" s="48" t="s">
+      <c r="D4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+      <c r="I4" s="52"/>
+      <c r="J4" s="52"/>
     </row>
     <row r="5" spans="2:11">
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
-      <c r="D5" s="50"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="51"/>
-      <c r="H5" s="51"/>
-      <c r="I5" s="51"/>
-      <c r="J5" s="51"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
     </row>
     <row r="6" spans="2:11" ht="32">
       <c r="B6" s="10" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="11"/>
-      <c r="D6" s="48" t="s">
+      <c r="D6" s="51" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
+      <c r="J6" s="52"/>
     </row>
     <row r="7" spans="2:11">
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
-      <c r="I7" s="51"/>
-      <c r="J7" s="51"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
     </row>
     <row r="8" spans="2:11" ht="33" customHeight="1">
       <c r="B8" s="10" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="11"/>
-      <c r="D8" s="52" t="s">
+      <c r="D8" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="53"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="54"/>
+      <c r="I8" s="54"/>
+      <c r="J8" s="54"/>
     </row>
     <row r="9" spans="2:11">
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
-      <c r="J9" s="51"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="44"/>
+      <c r="G9" s="44"/>
+      <c r="H9" s="44"/>
+      <c r="I9" s="44"/>
+      <c r="J9" s="44"/>
     </row>
     <row r="10" spans="2:11" ht="32">
       <c r="B10" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="11"/>
-      <c r="D10" s="54">
+      <c r="D10" s="46">
         <v>45995</v>
       </c>
-      <c r="E10" s="55"/>
-      <c r="F10" s="55"/>
-      <c r="G10" s="55"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="55"/>
-      <c r="J10" s="55"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
     </row>
     <row r="11" spans="2:11">
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
-      <c r="G11" s="51"/>
-      <c r="H11" s="51"/>
-      <c r="I11" s="51"/>
-      <c r="J11" s="51"/>
+      <c r="D11" s="43"/>
+      <c r="E11" s="44"/>
+      <c r="F11" s="44"/>
+      <c r="G11" s="44"/>
+      <c r="H11" s="44"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
     </row>
     <row r="12" spans="2:11" ht="31">
       <c r="B12" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C12" s="11"/>
-      <c r="D12" s="56">
-        <v>4</v>
-      </c>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
-      <c r="G12" s="51"/>
-      <c r="H12" s="51"/>
-      <c r="I12" s="51"/>
-      <c r="J12" s="51"/>
+      <c r="D12" s="45">
+        <v>5</v>
+      </c>
+      <c r="E12" s="44"/>
+      <c r="F12" s="44"/>
+      <c r="G12" s="44"/>
+      <c r="H12" s="44"/>
+      <c r="I12" s="44"/>
+      <c r="J12" s="44"/>
     </row>
     <row r="13" spans="2:11" ht="134" customHeight="1">
       <c r="B13" s="4"/>
@@ -1866,16 +1868,16 @@
       <c r="D13" s="4"/>
     </row>
     <row r="14" spans="2:11" ht="32">
-      <c r="B14" s="41"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="41"/>
-      <c r="F14" s="41"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="41"/>
-      <c r="J14" s="41"/>
-      <c r="K14" s="41"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1908,11 +1910,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -1979,9 +1981,15 @@
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="B9" s="15"/>
-      <c r="C9" s="16"/>
-      <c r="D9" s="17"/>
+      <c r="B9" s="15">
+        <v>5</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="B10" s="15"/>
@@ -2059,11 +2067,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="63">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
@@ -2092,7 +2100,7 @@
       <c r="C5" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="41" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2103,7 +2111,7 @@
       <c r="C6" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="D6" s="41" t="s">
         <v>21</v>
       </c>
     </row>
@@ -2114,7 +2122,7 @@
       <c r="C7" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="D7" s="46" t="s">
+      <c r="D7" s="41" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2125,7 +2133,7 @@
       <c r="C8" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="D8" s="46" t="s">
+      <c r="D8" s="41" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2136,7 +2144,7 @@
       <c r="C9" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="41" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2147,59 +2155,59 @@
       <c r="C10" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="D10" s="46" t="s">
+      <c r="D10" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="17">
       <c r="B11" s="20"/>
       <c r="C11" s="16"/>
-      <c r="D11" s="47"/>
+      <c r="D11" s="42"/>
     </row>
     <row r="12" spans="1:7" ht="17">
       <c r="B12" s="20"/>
       <c r="C12" s="16"/>
-      <c r="D12" s="47"/>
+      <c r="D12" s="42"/>
     </row>
     <row r="13" spans="1:7" ht="17">
       <c r="B13" s="20"/>
       <c r="C13" s="16"/>
-      <c r="D13" s="47"/>
+      <c r="D13" s="42"/>
     </row>
     <row r="14" spans="1:7" ht="17">
       <c r="B14" s="20"/>
       <c r="C14" s="16"/>
-      <c r="D14" s="47"/>
+      <c r="D14" s="42"/>
     </row>
     <row r="15" spans="1:7" ht="17">
       <c r="B15" s="20"/>
       <c r="C15" s="16"/>
-      <c r="D15" s="47"/>
+      <c r="D15" s="42"/>
     </row>
     <row r="16" spans="1:7" ht="17">
       <c r="B16" s="20"/>
       <c r="C16" s="16"/>
-      <c r="D16" s="47"/>
+      <c r="D16" s="42"/>
     </row>
     <row r="17" spans="2:4" ht="17">
       <c r="B17" s="20"/>
       <c r="C17" s="16"/>
-      <c r="D17" s="47"/>
+      <c r="D17" s="42"/>
     </row>
     <row r="18" spans="2:4" ht="17">
       <c r="B18" s="20"/>
       <c r="C18" s="16"/>
-      <c r="D18" s="47"/>
+      <c r="D18" s="42"/>
     </row>
     <row r="19" spans="2:4" ht="17">
       <c r="B19" s="20"/>
       <c r="C19" s="16"/>
-      <c r="D19" s="47"/>
+      <c r="D19" s="42"/>
     </row>
     <row r="20" spans="2:4" ht="17">
       <c r="B20" s="20"/>
       <c r="C20" s="16"/>
-      <c r="D20" s="47"/>
+      <c r="D20" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2230,14 +2238,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="60">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
     </row>
     <row r="3" spans="1:7">
       <c r="B3" s="21"/>
@@ -2554,14 +2562,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="60">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
     </row>
     <row r="3" spans="1:7">
       <c r="B3" s="21"/>
@@ -2810,14 +2818,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="60">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
     </row>
     <row r="3" spans="1:7">
       <c r="B3" s="21"/>
@@ -3198,15 +3206,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DC4784-38B4-904C-941F-7B874C5F62D5}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{533C6453-DD16-184C-B08A-36363D274383}">
   <dimension ref="A2:G28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
@@ -3219,14 +3218,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="60">
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
     </row>
     <row r="3" spans="1:7">
       <c r="B3" s="21"/>
@@ -3547,12 +3546,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0fe8f55b-6935-4298-952f-379117e6921e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="32ca420a-08c7-4d06-bbfa-5e08a735cd98" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3757,20 +3758,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0fe8f55b-6935-4298-952f-379117e6921e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="32ca420a-08c7-4d06-bbfa-5e08a735cd98" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7931E242-50D8-4124-8FCE-BD9D55441800}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{070B00FB-015B-4D7E-AC61-0F2BB9BDA9D9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0fe8f55b-6935-4298-952f-379117e6921e"/>
+    <ds:schemaRef ds:uri="32ca420a-08c7-4d06-bbfa-5e08a735cd98"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3795,12 +3797,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{070B00FB-015B-4D7E-AC61-0F2BB9BDA9D9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7931E242-50D8-4124-8FCE-BD9D55441800}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0fe8f55b-6935-4298-952f-379117e6921e"/>
-    <ds:schemaRef ds:uri="32ca420a-08c7-4d06-bbfa-5e08a735cd98"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>